<commit_message>
Actualizar tablas, scripts e imágenes
</commit_message>
<xml_diff>
--- a/results/supplementary/tables_submission/TableS2_community_assignments.xlsx
+++ b/results/supplementary/tables_submission/TableS2_community_assignments.xlsx
@@ -269,10 +269,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,32 +297,34 @@
       <family val="0"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Ubuntu"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Cambria"/>
+      <sz val="12"/>
+      <name val="Ubuntu"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Ubuntu"/>
       <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF2E4057"/>
-        <bgColor rgb="FF333399"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor rgb="FFFFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -365,20 +368,28 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -391,66 +402,6 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="FF000000"/>
-      <rgbColor rgb="FFFFFFFF"/>
-      <rgbColor rgb="FFFF0000"/>
-      <rgbColor rgb="FF00FF00"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008000"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FF808000"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
-      <rgbColor rgb="FF808080"/>
-      <rgbColor rgb="FF9999FF"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFF2F2F2"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FF660066"/>
-      <rgbColor rgb="FFFF8080"/>
-      <rgbColor rgb="FF0066CC"/>
-      <rgbColor rgb="FFCCCCFF"/>
-      <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFFF00FF"/>
-      <rgbColor rgb="FFFFFF00"/>
-      <rgbColor rgb="FF00FFFF"/>
-      <rgbColor rgb="FF800080"/>
-      <rgbColor rgb="FF800000"/>
-      <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FF0000FF"/>
-      <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
-      <rgbColor rgb="FFFFFF99"/>
-      <rgbColor rgb="FF99CCFF"/>
-      <rgbColor rgb="FFFF99CC"/>
-      <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFFFCC99"/>
-      <rgbColor rgb="FF3366FF"/>
-      <rgbColor rgb="FF33CCCC"/>
-      <rgbColor rgb="FF99CC00"/>
-      <rgbColor rgb="FFFFCC00"/>
-      <rgbColor rgb="FFFF9900"/>
-      <rgbColor rgb="FFFF6600"/>
-      <rgbColor rgb="FF666699"/>
-      <rgbColor rgb="FF969696"/>
-      <rgbColor rgb="FF003366"/>
-      <rgbColor rgb="FF339966"/>
-      <rgbColor rgb="FF003300"/>
-      <rgbColor rgb="FF333300"/>
-      <rgbColor rgb="FF993300"/>
-      <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FF333399"/>
-      <rgbColor rgb="FF2E4057"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -635,67 +586,68 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H42"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.58984375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="13"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="1" width="8.59"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E2" s="2" t="n">
+      <c r="D2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="F2" s="2" t="n">
+      <c r="F2" s="5" t="n">
         <v>0.0692</v>
       </c>
-      <c r="G2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2" t="n">
+      <c r="G2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -703,51 +655,51 @@
       <c r="A3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="3" t="n">
+      <c r="D3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="F3" s="5" t="n">
         <v>0.0128</v>
       </c>
-      <c r="G3" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" s="3" t="n">
+      <c r="G3" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="2" t="n">
+      <c r="D4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="5" t="n">
         <v>0.0256</v>
       </c>
-      <c r="G4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" s="2" t="n">
+      <c r="G4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -755,51 +707,51 @@
       <c r="A5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="3" t="n">
+      <c r="D5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="3" t="n">
+      <c r="F5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="2" t="n">
+      <c r="D6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="5" t="n">
         <v>0.0051</v>
       </c>
-      <c r="G6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="2" t="n">
+      <c r="G6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -807,51 +759,51 @@
       <c r="A7" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="3" t="n">
+      <c r="D7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="F7" s="5" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="3" t="n">
+      <c r="G7" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="2" t="n">
+      <c r="E8" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="F8" s="2" t="n">
+      <c r="F8" s="5" t="n">
         <v>0.0385</v>
       </c>
-      <c r="G8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="2" t="n">
+      <c r="G8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -859,51 +811,51 @@
       <c r="A9" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="3" t="n">
+      <c r="E9" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="F9" s="5" t="n">
         <v>0.0654</v>
       </c>
-      <c r="G9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="3" t="n">
+      <c r="G9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="2" t="n">
+      <c r="D10" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="2" t="n">
+      <c r="E10" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="2" t="n">
+      <c r="F10" s="5" t="n">
         <v>0.0013</v>
       </c>
-      <c r="G10" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2" t="n">
+      <c r="G10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -911,51 +863,51 @@
       <c r="A11" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="3" t="n">
+      <c r="E11" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="F11" s="5" t="n">
         <v>0.0321</v>
       </c>
-      <c r="G11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="3" t="n">
+      <c r="G11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="2" t="n">
+      <c r="D12" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="2" t="n">
+      <c r="E12" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="5" t="n">
         <v>0.0333</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="2" t="n">
+      <c r="G12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H12" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -963,51 +915,51 @@
       <c r="A13" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="B13" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="3" t="n">
+      <c r="E13" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="F13" s="5" t="n">
         <v>0.0269</v>
       </c>
-      <c r="G13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="3" t="n">
+      <c r="G13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="2" t="n">
+      <c r="E14" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="F14" s="2" t="n">
+      <c r="F14" s="5" t="n">
         <v>0.0026</v>
       </c>
-      <c r="G14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" s="2" t="n">
+      <c r="G14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1015,51 +967,51 @@
       <c r="A15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E15" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="F15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" s="3" t="n">
+      <c r="F15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D16" s="2" t="n">
+      <c r="D16" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="2" t="n">
+      <c r="E16" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="F16" s="2" t="n">
+      <c r="F16" s="5" t="n">
         <v>0.0141</v>
       </c>
-      <c r="G16" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="2" t="n">
+      <c r="G16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1067,51 +1019,51 @@
       <c r="A17" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B17" s="3" t="s">
+      <c r="B17" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E17" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="F17" s="3" t="n">
+      <c r="F17" s="5" t="n">
         <v>0.0026</v>
       </c>
-      <c r="G17" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H17" s="3" t="n">
+      <c r="G17" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D18" s="2" t="n">
+      <c r="D18" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="2" t="n">
+      <c r="E18" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="2" t="n">
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1119,51 +1071,51 @@
       <c r="A19" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="B19" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E19" s="3" t="n">
+      <c r="E19" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="F19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="3" t="n">
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
+      <c r="A20" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D20" s="2" t="n">
+      <c r="D20" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E20" s="2" t="n">
+      <c r="E20" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="F20" s="2" t="n">
+      <c r="F20" s="5" t="n">
         <v>0.041</v>
       </c>
-      <c r="G20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H20" s="2" t="n">
+      <c r="G20" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1171,51 +1123,51 @@
       <c r="A21" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="F21" s="5" t="n">
         <v>0.0333</v>
       </c>
-      <c r="G21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H21" s="3" t="n">
+      <c r="G21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="2" t="n">
+      <c r="D22" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E22" s="2" t="n">
+      <c r="E22" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="F22" s="2" t="n">
+      <c r="F22" s="5" t="n">
         <v>0.0346</v>
       </c>
-      <c r="G22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="2" t="n">
+      <c r="G22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1223,51 +1175,51 @@
       <c r="A23" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E23" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="F23" s="3" t="n">
+      <c r="F23" s="5" t="n">
         <v>0.0051</v>
       </c>
-      <c r="G23" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H23" s="3" t="n">
+      <c r="G23" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D24" s="2" t="n">
+      <c r="D24" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E24" s="2" t="n">
+      <c r="E24" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H24" s="2" t="n">
+      <c r="F24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1275,51 +1227,51 @@
       <c r="A25" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="B25" s="3" t="s">
+      <c r="B25" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E25" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H25" s="3" t="n">
+      <c r="F25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="2" t="n">
+      <c r="D26" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E26" s="2" t="n">
+      <c r="E26" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="F26" s="2" t="n">
+      <c r="F26" s="5" t="n">
         <v>0.1077</v>
       </c>
-      <c r="G26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H26" s="2" t="n">
+      <c r="G26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1327,51 +1279,51 @@
       <c r="A27" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B27" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E27" s="3" t="n">
+      <c r="E27" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F27" s="3" t="n">
+      <c r="F27" s="5" t="n">
         <v>0.0321</v>
       </c>
-      <c r="G27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H27" s="3" t="n">
+      <c r="G27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
+      <c r="A28" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="B28" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C28" s="2" t="s">
+      <c r="C28" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D28" s="2" t="n">
+      <c r="D28" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="E28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H28" s="2" t="n">
+      <c r="E28" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1379,51 +1331,51 @@
       <c r="A29" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="E29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G29" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H29" s="3" t="n">
+      <c r="E29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
+      <c r="A30" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B30" s="2" t="s">
+      <c r="B30" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C30" s="2" t="s">
+      <c r="C30" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D30" s="2" t="n">
+      <c r="D30" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="E30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="2" t="n">
+      <c r="E30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1431,51 +1383,51 @@
       <c r="A31" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="3" t="s">
+      <c r="C31" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D31" s="3" t="n">
+      <c r="D31" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="E31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G31" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="3" t="n">
+      <c r="E31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
+      <c r="A32" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="B32" s="2" t="s">
+      <c r="B32" s="4" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="2" t="s">
+      <c r="C32" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D32" s="2" t="n">
+      <c r="D32" s="4" t="n">
         <v>9</v>
       </c>
-      <c r="E32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H32" s="2" t="n">
+      <c r="E32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1483,51 +1435,51 @@
       <c r="A33" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C33" s="3" t="s">
+      <c r="C33" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D33" s="3" t="n">
+      <c r="D33" s="4" t="n">
         <v>10</v>
       </c>
-      <c r="E33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H33" s="3" t="n">
+      <c r="E33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="2" t="s">
+      <c r="A34" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B34" s="2" t="s">
+      <c r="B34" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C34" s="2" t="s">
+      <c r="C34" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D34" s="2" t="n">
+      <c r="D34" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="E34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H34" s="2" t="n">
+      <c r="E34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1535,51 +1487,51 @@
       <c r="A35" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="B35" s="3" t="s">
+      <c r="B35" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C35" s="3" t="s">
+      <c r="C35" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D35" s="3" t="n">
+      <c r="D35" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="E35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G35" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H35" s="3" t="n">
+      <c r="E35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="2" t="s">
+      <c r="A36" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="B36" s="2" t="s">
+      <c r="B36" s="4" t="s">
         <v>69</v>
       </c>
-      <c r="C36" s="2" t="s">
+      <c r="C36" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D36" s="2" t="n">
+      <c r="D36" s="4" t="n">
         <v>13</v>
       </c>
-      <c r="E36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H36" s="2" t="n">
+      <c r="E36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1587,51 +1539,51 @@
       <c r="A37" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="C37" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D37" s="3" t="n">
+      <c r="D37" s="4" t="n">
         <v>14</v>
       </c>
-      <c r="E37" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G37" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H37" s="3" t="n">
+      <c r="E37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2" t="s">
+      <c r="A38" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B38" s="2" t="s">
+      <c r="B38" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="C38" s="2" t="s">
+      <c r="C38" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D38" s="2" t="n">
+      <c r="D38" s="4" t="n">
         <v>15</v>
       </c>
-      <c r="E38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G38" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="2" t="n">
+      <c r="E38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1639,51 +1591,51 @@
       <c r="A39" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B39" s="3" t="s">
+      <c r="B39" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C39" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D39" s="3" t="n">
+      <c r="D39" s="4" t="n">
         <v>16</v>
       </c>
-      <c r="E39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H39" s="3" t="n">
+      <c r="E39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
+      <c r="A40" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B40" s="2" t="s">
+      <c r="B40" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D40" s="2" t="n">
+      <c r="D40" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="E40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="2" t="n">
+      <c r="E40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1691,51 +1643,51 @@
       <c r="A41" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B41" s="3" t="s">
+      <c r="B41" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="C41" s="3" t="s">
+      <c r="C41" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D41" s="3" t="n">
+      <c r="D41" s="4" t="n">
         <v>18</v>
       </c>
-      <c r="E41" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F41" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G41" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H41" s="3" t="n">
+      <c r="E41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="4" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="C42" s="2" t="s">
+      <c r="C42" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D42" s="2" t="n">
+      <c r="D42" s="4" t="n">
         <v>19</v>
       </c>
-      <c r="E42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="2" t="n">
+      <c r="E42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="4" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>